<commit_message>
Update tooth wear from corrected file
- Reprocess new BWE_Tooth_Wear_rate.xlsx (user fixed length outliers)
- Handle SMU/age=0 as fresh-install (not error): 29 fresh cells skipped
  in wear-rate calc, not counted against data quality
- Refresh embedded wear timeline (22 inspections) and weighted wear rates
  (hottest tooth T9 2.56 cm/1000hr, bucket B1 3.05)
- Regenerate sheet-template/BWE_Tooth_Wear_clean.xlsx + wear.csv
- 4 remaining issues (T7 B7 = 28cm in 4 sheets) noted for user

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL3E7XjWGCNSS7seQn2heL
</commit_message>
<xml_diff>
--- a/sheet-template/BWE_Tooth_Wear_clean.xlsx
+++ b/sheet-template/BWE_Tooth_Wear_clean.xlsx
@@ -517,7 +517,7 @@
         <v>6605</v>
       </c>
       <c r="D3" t="n">
-        <v>18.16</v>
+        <v>18.11</v>
       </c>
       <c r="E3" t="n">
         <v>25.15</v>
@@ -547,7 +547,7 @@
         <v>6605</v>
       </c>
       <c r="D4" t="n">
-        <v>18.2</v>
+        <v>18.19</v>
       </c>
       <c r="E4" t="n">
         <v>25.17</v>
@@ -559,7 +559,7 @@
         <v>16.5</v>
       </c>
       <c r="H4" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="5">
@@ -637,7 +637,7 @@
         <v>6997</v>
       </c>
       <c r="D7" t="n">
-        <v>18</v>
+        <v>17.99</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -667,7 +667,7 @@
         <v>7065</v>
       </c>
       <c r="D8" t="n">
-        <v>18</v>
+        <v>17.99</v>
       </c>
       <c r="E8" t="n">
         <v>25.01</v>
@@ -697,7 +697,7 @@
         <v>7141</v>
       </c>
       <c r="D9" t="n">
-        <v>18.07</v>
+        <v>18.06</v>
       </c>
       <c r="E9" t="n">
         <v>25.33</v>
@@ -727,7 +727,7 @@
         <v>7190</v>
       </c>
       <c r="D10" t="n">
-        <v>18.14</v>
+        <v>18.12</v>
       </c>
       <c r="E10" t="n">
         <v>25.47</v>
@@ -757,7 +757,7 @@
         <v>7190</v>
       </c>
       <c r="D11" t="n">
-        <v>18.14</v>
+        <v>18.13</v>
       </c>
       <c r="E11" t="n">
         <v>25.56</v>
@@ -787,7 +787,7 @@
         <v>7254</v>
       </c>
       <c r="D12" t="n">
-        <v>18.19</v>
+        <v>18.17</v>
       </c>
       <c r="E12" t="n">
         <v>25.78</v>
@@ -817,7 +817,7 @@
         <v>7319</v>
       </c>
       <c r="D13" t="n">
-        <v>18.28</v>
+        <v>18.27</v>
       </c>
       <c r="E13" t="n">
         <v>26.08</v>
@@ -847,7 +847,7 @@
         <v>7377</v>
       </c>
       <c r="D14" t="n">
-        <v>18.33</v>
+        <v>18.32</v>
       </c>
       <c r="E14" t="n">
         <v>26.11</v>
@@ -877,7 +877,7 @@
         <v>7440</v>
       </c>
       <c r="D15" t="n">
-        <v>18.44</v>
+        <v>18.43</v>
       </c>
       <c r="E15" t="n">
         <v>26.13</v>
@@ -907,7 +907,7 @@
         <v>7471</v>
       </c>
       <c r="D16" t="n">
-        <v>18.44</v>
+        <v>18.43</v>
       </c>
       <c r="E16" t="n">
         <v>26.2</v>
@@ -937,7 +937,7 @@
         <v>7525</v>
       </c>
       <c r="D17" t="n">
-        <v>18.52</v>
+        <v>18.46</v>
       </c>
       <c r="E17" t="n">
         <v>26.38</v>
@@ -967,7 +967,7 @@
         <v>7558</v>
       </c>
       <c r="D18" t="n">
-        <v>18.53</v>
+        <v>18.47</v>
       </c>
       <c r="E18" t="n">
         <v>26.38</v>
@@ -997,7 +997,7 @@
         <v>7612</v>
       </c>
       <c r="D19" t="n">
-        <v>18.57</v>
+        <v>18.51</v>
       </c>
       <c r="E19" t="n">
         <v>26.42</v>
@@ -1027,7 +1027,7 @@
         <v>7670</v>
       </c>
       <c r="D20" t="n">
-        <v>18.53</v>
+        <v>18.47</v>
       </c>
       <c r="E20" t="n">
         <v>26.42</v>
@@ -1057,7 +1057,7 @@
         <v>7727</v>
       </c>
       <c r="D21" t="n">
-        <v>18.53</v>
+        <v>18.47</v>
       </c>
       <c r="E21" t="n">
         <v>26.42</v>
@@ -1087,7 +1087,7 @@
         <v>7777</v>
       </c>
       <c r="D22" t="n">
-        <v>18.6</v>
+        <v>18.54</v>
       </c>
       <c r="E22" t="n">
         <v>26.58</v>
@@ -1117,7 +1117,7 @@
         <v>7777</v>
       </c>
       <c r="D23" t="n">
-        <v>18.6</v>
+        <v>18.54</v>
       </c>
       <c r="E23" t="n">
         <v>26.58</v>

</xml_diff>

<commit_message>
Rebrand to BWE Performance Record + header restructure
- Rename product 'BWE Tooth Intelligence/Record' -> 'BWE Performance Record'
  everywhere (title, hero heading, sticky header, report title, preview)
- Remove 'Fleet Intelligence Dashboard' subtitle from hero and 'Tooth
  Intelligence' from the topbar chip; hero subtitle is now the desc block
- Move ITD org logo to the top-LEFT of the sticky header (flip border)
- Loss-cost bar chart bars thinned via barThickness/barPercentage so a
  handful of days doesn't fill the whole panel with wide bars
- Refresh embedded wear data + rates from new xlsx (0 errors this time)

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL3E7XjWGCNSS7seQn2heL
</commit_message>
<xml_diff>
--- a/sheet-template/BWE_Tooth_Wear_clean.xlsx
+++ b/sheet-template/BWE_Tooth_Wear_clean.xlsx
@@ -487,7 +487,7 @@
         <v>6567</v>
       </c>
       <c r="D2" t="n">
-        <v>18.16</v>
+        <v>18.11</v>
       </c>
       <c r="E2" t="n">
         <v>25.15</v>
@@ -547,7 +547,7 @@
         <v>6605</v>
       </c>
       <c r="D4" t="n">
-        <v>18.19</v>
+        <v>18.15</v>
       </c>
       <c r="E4" t="n">
         <v>25.17</v>
@@ -577,7 +577,7 @@
         <v>6659</v>
       </c>
       <c r="D5" t="n">
-        <v>18.22</v>
+        <v>18.17</v>
       </c>
       <c r="E5" t="n">
         <v>25.17</v>
@@ -607,7 +607,7 @@
         <v>6786</v>
       </c>
       <c r="D6" t="n">
-        <v>18.27</v>
+        <v>18.22</v>
       </c>
       <c r="E6" t="n">
         <v>25.32</v>

</xml_diff>